<commit_message>
test: strengthen excel import approval coverage
</commit_message>
<xml_diff>
--- a/backend/data/import_samples/listino_test.xlsx
+++ b/backend/data/import_samples/listino_test.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bicchiere Acqua 200ml Pet x100</t>
+          <t>BICCHIERE ACQUA 200ML BIANCO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">

</xml_diff>